<commit_message>
Update Alphabet, ServiceNow, Cheniere and Altria models for Q3 results
Alphabet: higher 2027 to 2028 reinvestment for the capex guide; base 250.
ServiceNow: net debt and share count after Armis; base 110.
Cheniere: raised 2026 guidance, lower net debt; base 380.
Altria: share count after buybacks; base 66.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkHMtTWpPSAxFWhvppEUAQ
</commit_message>
<xml_diff>
--- a/models/holdings/GOOG_Valuation.xlsx
+++ b/models/holdings/GOOG_Valuation.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="127">
   <si>
     <t xml:space="preserve">Alphabet (GOOG): valuation summary</t>
   </si>
@@ -90,15 +90,12 @@
     <t xml:space="preserve">Share price ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 23, 2026 intraday (Yahoo Finance via the site's price feed)</t>
+    <t xml:space="preserve">Oct 28, 2026 close (before Q3 results)</t>
   </si>
   <si>
     <t xml:space="preserve">Price date</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 23, 2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Text</t>
   </si>
   <si>
@@ -117,7 +114,7 @@
     <t xml:space="preserve">Other non-operating assets, less outside claims</t>
   </si>
   <si>
-    <t xml:space="preserve">Private stakes (SpaceX, Anthropic, others) excluded</t>
+    <t xml:space="preserve">Private stakes (SpaceX, Anthropic, others) excluded; Q3 included an $8.2B unrealized loss on SpaceX</t>
   </si>
   <si>
     <t xml:space="preserve">Tax rate</t>
@@ -141,7 +138,7 @@
     <t xml:space="preserve">Base-year revenue (2026E)</t>
   </si>
   <si>
-    <t xml:space="preserve">2026E consensus $499.6B (Stock Analysis)</t>
+    <t xml:space="preserve">2026E consensus $499.6B (Stock Analysis). Q3 2026: revenue $127.6B, capex $51.4B, free cash flow -$9.1B. Reinvestment raised Oct 29, 2026 for 2027 capex guided to rise significantly from $195B to $205B</t>
   </si>
   <si>
     <t xml:space="preserve">Selected scenario (1 Bear, 2 Base, 3 Bull)</t>
@@ -243,7 +240,7 @@
     <t xml:space="preserve">Value vs share price</t>
   </si>
   <si>
-    <t xml:space="preserve">Base: Cloud and Search grow, capex peaks 2027</t>
+    <t xml:space="preserve">Base: Cloud and Search grow, capex peaks 2027 to 2028</t>
   </si>
   <si>
     <t xml:space="preserve">Bull: Cloud and AI monetization compound</t>
@@ -926,7 +923,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
@@ -985,7 +982,7 @@
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">GOOG!B4</f>
-        <v>320.47</v>
+        <v>321.89</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">GOOG!B10</f>
@@ -993,27 +990,27 @@
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">GOOG!B75</f>
-        <v>149.10637041906</v>
+        <v>132.552074944012</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">GOOG!B76</f>
-        <v>267.306138447792</v>
+        <v>252.467499447734</v>
       </c>
       <c r="G5" s="5" t="n">
         <f aca="false">GOOG!B77</f>
-        <v>343.939756647134</v>
+        <v>335.030538938902</v>
       </c>
       <c r="H5" s="7" t="n">
         <f aca="false">F5/C5-1</f>
-        <v>-0.165893411402652</v>
+        <v>-0.215671504402951</v>
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">GOOG!B86</f>
-        <v>0.0843278176794784</v>
+        <v>0.082000599052872</v>
       </c>
       <c r="J5" s="8" t="n">
         <f aca="false">IF(F5&lt;10,ROUND(F5*4,0)/4,IF(F5&lt;100,ROUND(F5,0),ROUND(F5/5,0)*5))</f>
-        <v>265</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1026,7 +1023,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1034,7 +1031,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1042,7 +1039,7 @@
         <v>16</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1059,12 +1056,6 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1105,7 +1096,7 @@
         <v>21</v>
       </c>
       <c r="B4" s="10" t="n">
-        <v>320.47</v>
+        <v>321.89</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>22</v>
@@ -1116,142 +1107,142 @@
         <v>23</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>12.23</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>140</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="B7" s="13" t="n">
-        <v>121.68</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>0.17</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B10" s="15" t="n">
         <f aca="false">WACC!B29</f>
         <v>0.0922</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="B11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" s="13" t="n">
         <v>499.6</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="C15" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="D15" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="E15" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="F15" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="G15" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="H15" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="H15" s="17" t="s">
+      <c r="I15" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="J15" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="J15" s="17" t="s">
+      <c r="K15" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="K15" s="17" t="s">
+      <c r="L15" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="L15" s="9" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.5</v>
@@ -1295,7 +1286,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0</v>
@@ -1330,7 +1321,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -1346,7 +1337,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B20" s="13" t="n">
         <v>565</v>
@@ -1390,7 +1381,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">B20/$B$12-1</f>
@@ -1438,38 +1429,38 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B22" s="22" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="C22" s="22" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="D22" s="22" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="E22" s="22" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="F22" s="22" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="G22" s="7" t="n">
         <f aca="false">$F22+($L22-$F22)*G$17/5</f>
-        <v>0.286</v>
+        <v>0.278</v>
       </c>
       <c r="H22" s="7" t="n">
         <f aca="false">$F22+($L22-$F22)*H$17/5</f>
-        <v>0.282</v>
+        <v>0.276</v>
       </c>
       <c r="I22" s="7" t="n">
         <f aca="false">$F22+($L22-$F22)*I$17/5</f>
-        <v>0.278</v>
+        <v>0.274</v>
       </c>
       <c r="J22" s="7" t="n">
         <f aca="false">$F22+($L22-$F22)*J$17/5</f>
-        <v>0.274</v>
+        <v>0.272</v>
       </c>
       <c r="K22" s="7" t="n">
         <f aca="false">$F22+($L22-$F22)*K$17/5</f>
@@ -1481,43 +1472,43 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">B20*B22</f>
-        <v>169.5</v>
+        <v>163.85</v>
       </c>
       <c r="C23" s="20" t="n">
         <f aca="false">C20*C22</f>
-        <v>176.9</v>
+        <v>170.8</v>
       </c>
       <c r="D23" s="20" t="n">
         <f aca="false">D20*D22</f>
-        <v>188.5</v>
+        <v>182</v>
       </c>
       <c r="E23" s="20" t="n">
         <f aca="false">E20*E22</f>
-        <v>200.1</v>
+        <v>193.2</v>
       </c>
       <c r="F23" s="20" t="n">
         <f aca="false">F20*F22</f>
-        <v>210.25</v>
+        <v>203</v>
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">G20*G22</f>
-        <v>217.215652898551</v>
+        <v>211.13969057971</v>
       </c>
       <c r="H23" s="20" t="n">
         <f aca="false">H20*H22</f>
-        <v>223.694610022495</v>
+        <v>218.935150234783</v>
       </c>
       <c r="I23" s="20" t="n">
         <f aca="false">I20*I22</f>
-        <v>229.626943255768</v>
+        <v>226.322958460721</v>
       </c>
       <c r="J23" s="20" t="n">
         <f aca="false">J20*J22</f>
-        <v>234.956031310991</v>
+        <v>233.241023783174</v>
       </c>
       <c r="K23" s="20" t="n">
         <f aca="false">K20*K22</f>
@@ -1530,43 +1521,43 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B24" s="20" t="n">
         <f aca="false">B23*(1-$B$9)</f>
-        <v>140.685</v>
+        <v>135.9955</v>
       </c>
       <c r="C24" s="20" t="n">
         <f aca="false">C23*(1-$B$9)</f>
-        <v>146.827</v>
+        <v>141.764</v>
       </c>
       <c r="D24" s="20" t="n">
         <f aca="false">D23*(1-$B$9)</f>
-        <v>156.455</v>
+        <v>151.06</v>
       </c>
       <c r="E24" s="20" t="n">
         <f aca="false">E23*(1-$B$9)</f>
-        <v>166.083</v>
+        <v>160.356</v>
       </c>
       <c r="F24" s="20" t="n">
         <f aca="false">F23*(1-$B$9)</f>
-        <v>174.5075</v>
+        <v>168.49</v>
       </c>
       <c r="G24" s="20" t="n">
         <f aca="false">G23*(1-$B$9)</f>
-        <v>180.288991905797</v>
+        <v>175.245943181159</v>
       </c>
       <c r="H24" s="20" t="n">
         <f aca="false">H23*(1-$B$9)</f>
-        <v>185.666526318671</v>
+        <v>181.71617469487</v>
       </c>
       <c r="I24" s="20" t="n">
         <f aca="false">I23*(1-$B$9)</f>
-        <v>190.590362902288</v>
+        <v>187.848055522399</v>
       </c>
       <c r="J24" s="20" t="n">
         <f aca="false">J23*(1-$B$9)</f>
-        <v>195.013505988123</v>
+        <v>193.590049740034</v>
       </c>
       <c r="K24" s="20" t="n">
         <f aca="false">K23*(1-$B$9)</f>
@@ -1579,38 +1570,38 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B25" s="22" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="C25" s="22" t="n">
-        <v>0.19</v>
+        <v>0.28</v>
       </c>
       <c r="D25" s="22" t="n">
-        <v>0.14</v>
+        <v>0.21</v>
       </c>
       <c r="E25" s="22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F25" s="22" t="n">
         <v>0.11</v>
-      </c>
-      <c r="F25" s="22" t="n">
-        <v>0.09</v>
       </c>
       <c r="G25" s="7" t="n">
         <f aca="false">$F25+($L25-$F25)*G$17/5</f>
-        <v>0.084</v>
+        <v>0.1</v>
       </c>
       <c r="H25" s="7" t="n">
         <f aca="false">$F25+($L25-$F25)*H$17/5</f>
-        <v>0.078</v>
+        <v>0.09</v>
       </c>
       <c r="I25" s="7" t="n">
         <f aca="false">$F25+($L25-$F25)*I$17/5</f>
-        <v>0.072</v>
+        <v>0.08</v>
       </c>
       <c r="J25" s="7" t="n">
         <f aca="false">$F25+($L25-$F25)*J$17/5</f>
-        <v>0.066</v>
+        <v>0.07</v>
       </c>
       <c r="K25" s="7" t="n">
         <f aca="false">$F25+($L25-$F25)*K$17/5</f>
@@ -1622,43 +1613,43 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B26" s="20" t="n">
         <f aca="false">B20*B25</f>
-        <v>135.6</v>
+        <v>192.1</v>
       </c>
       <c r="C26" s="20" t="n">
         <f aca="false">C20*C25</f>
-        <v>115.9</v>
+        <v>170.8</v>
       </c>
       <c r="D26" s="20" t="n">
         <f aca="false">D20*D25</f>
-        <v>91</v>
+        <v>136.5</v>
       </c>
       <c r="E26" s="20" t="n">
         <f aca="false">E20*E25</f>
-        <v>75.9</v>
+        <v>103.5</v>
       </c>
       <c r="F26" s="20" t="n">
         <f aca="false">F20*F25</f>
-        <v>65.25</v>
+        <v>79.75</v>
       </c>
       <c r="G26" s="20" t="n">
         <f aca="false">G20*G25</f>
-        <v>63.7976043478261</v>
+        <v>75.9495289855073</v>
       </c>
       <c r="H26" s="20" t="n">
         <f aca="false">H20*H25</f>
-        <v>61.8729772402647</v>
+        <v>71.39189681569</v>
       </c>
       <c r="I26" s="20" t="n">
         <f aca="false">I20*I25</f>
-        <v>59.4717263108465</v>
+        <v>66.0796959009405</v>
       </c>
       <c r="J26" s="20" t="n">
         <f aca="false">J20*J25</f>
-        <v>56.595248417976</v>
+        <v>60.0252634736109</v>
       </c>
       <c r="K26" s="20" t="n">
         <f aca="false">K20*K25</f>
@@ -1671,7 +1662,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B27" s="20" t="n">
         <f aca="false">$B$11*(B20-$B$12)</f>
@@ -1720,43 +1711,43 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B28" s="20" t="n">
         <f aca="false">B24-B26-B27</f>
-        <v>5.08500000000001</v>
+        <v>-56.1045</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">C24-C26-C27</f>
-        <v>30.927</v>
+        <v>-29.036</v>
       </c>
       <c r="D28" s="20" t="n">
         <f aca="false">D24-D26-D27</f>
-        <v>65.455</v>
+        <v>14.56</v>
       </c>
       <c r="E28" s="20" t="n">
         <f aca="false">E24-E26-E27</f>
-        <v>90.183</v>
+        <v>56.856</v>
       </c>
       <c r="F28" s="20" t="n">
         <f aca="false">F24-F26-F27</f>
-        <v>109.2575</v>
+        <v>88.74</v>
       </c>
       <c r="G28" s="20" t="n">
         <f aca="false">G24-G26-G27</f>
-        <v>116.491387557971</v>
+        <v>99.2964141956522</v>
       </c>
       <c r="H28" s="20" t="n">
         <f aca="false">H24-H26-H27</f>
-        <v>123.793549078406</v>
+        <v>110.32427787918</v>
       </c>
       <c r="I28" s="20" t="n">
         <f aca="false">I24-I26-I27</f>
-        <v>131.118636591441</v>
+        <v>121.768359621458</v>
       </c>
       <c r="J28" s="20" t="n">
         <f aca="false">J24-J26-J27</f>
-        <v>138.418257570147</v>
+        <v>133.564786266423</v>
       </c>
       <c r="K28" s="20" t="n">
         <f aca="false">K24-K26-K27</f>
@@ -1769,7 +1760,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B29" s="23" t="n">
         <f aca="false">1/(1+$B$10)^B$16</f>
@@ -1814,43 +1805,43 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B30" s="20" t="n">
         <f aca="false">B28*B29</f>
-        <v>4.86563885776903</v>
+        <v>-53.6842153973849</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">C28*C29</f>
-        <v>27.0947118099113</v>
+        <v>-25.4380331785361</v>
       </c>
       <c r="D30" s="20" t="n">
         <f aca="false">D28*D29</f>
-        <v>52.5033961875651</v>
+        <v>11.6790076921694</v>
       </c>
       <c r="E30" s="20" t="n">
         <f aca="false">E28*E29</f>
-        <v>66.2318789165653</v>
+        <v>41.7559818112087</v>
       </c>
       <c r="F30" s="20" t="n">
         <f aca="false">F28*F29</f>
-        <v>73.4668609556003</v>
+        <v>59.6704962240576</v>
       </c>
       <c r="G30" s="20" t="n">
         <f aca="false">G28*G29</f>
-        <v>71.7186112236053</v>
+        <v>61.1324242494077</v>
       </c>
       <c r="H30" s="20" t="n">
         <f aca="false">H28*H29</f>
-        <v>69.7804707196737</v>
+        <v>62.1880550281444</v>
       </c>
       <c r="I30" s="20" t="n">
         <f aca="false">I28*I29</f>
-        <v>67.6703048840911</v>
+        <v>62.8446286129061</v>
       </c>
       <c r="J30" s="20" t="n">
         <f aca="false">J28*J29</f>
-        <v>65.4071030627145</v>
+        <v>63.1136809134457</v>
       </c>
       <c r="K30" s="20" t="n">
         <f aca="false">K28*K29</f>
@@ -1860,7 +1851,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B31" s="20" t="n">
         <f aca="false">L28/($B$10-L21)</f>
@@ -1873,7 +1864,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B32" s="20" t="n">
         <f aca="false">B31/(1+$B$10)^$K$16</f>
@@ -1882,34 +1873,34 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B33" s="20" t="n">
         <f aca="false">SUM(B30:K30)+B32+$B$7+$B$8</f>
-        <v>1823.5709102251</v>
+        <v>1626.41395956302</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B34" s="24" t="n">
         <f aca="false">B33/$B$6</f>
-        <v>149.10637041906</v>
+        <v>132.552074944012</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B35" s="7" t="n">
         <f aca="false">B34/$B$4-1</f>
-        <v>-0.534725963681281</v>
+        <v>-0.588206918686471</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B37" s="19"/>
       <c r="C37" s="19"/>
@@ -1925,7 +1916,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B38" s="13" t="n">
         <v>600</v>
@@ -1969,7 +1960,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" s="7" t="n">
         <f aca="false">B38/$B$12-1</f>
@@ -2017,38 +2008,38 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B40" s="22" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="C40" s="22" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="D40" s="22" t="n">
         <v>0.33</v>
       </c>
-      <c r="C40" s="22" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="D40" s="22" t="n">
-        <v>0.34</v>
-      </c>
       <c r="E40" s="22" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="F40" s="22" t="n">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="G40" s="7" t="n">
         <f aca="false">$F40+($L40-$F40)*G$17/5</f>
-        <v>0.336</v>
+        <v>0.328</v>
       </c>
       <c r="H40" s="7" t="n">
         <f aca="false">$F40+($L40-$F40)*H$17/5</f>
-        <v>0.332</v>
+        <v>0.326</v>
       </c>
       <c r="I40" s="7" t="n">
         <f aca="false">$F40+($L40-$F40)*I$17/5</f>
-        <v>0.328</v>
+        <v>0.324</v>
       </c>
       <c r="J40" s="7" t="n">
         <f aca="false">$F40+($L40-$F40)*J$17/5</f>
-        <v>0.324</v>
+        <v>0.322</v>
       </c>
       <c r="K40" s="7" t="n">
         <f aca="false">$F40+($L40-$F40)*K$17/5</f>
@@ -2060,43 +2051,43 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B41" s="20" t="n">
         <f aca="false">B38*B40</f>
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C41" s="20" t="n">
         <f aca="false">C38*C40</f>
-        <v>231.15</v>
+        <v>224.25</v>
       </c>
       <c r="D41" s="20" t="n">
         <f aca="false">D38*D40</f>
-        <v>261.8</v>
+        <v>254.1</v>
       </c>
       <c r="E41" s="20" t="n">
         <f aca="false">E38*E40</f>
-        <v>287.3</v>
+        <v>278.85</v>
       </c>
       <c r="F41" s="20" t="n">
         <f aca="false">F38*F40</f>
-        <v>311.1</v>
+        <v>301.95</v>
       </c>
       <c r="G41" s="20" t="n">
         <f aca="false">G38*G40</f>
-        <v>330.274241893491</v>
+        <v>322.410569467456</v>
       </c>
       <c r="H41" s="20" t="n">
         <f aca="false">H38*H40</f>
-        <v>347.784453447787</v>
+        <v>341.499192240899</v>
       </c>
       <c r="I41" s="20" t="n">
         <f aca="false">I38*I40</f>
-        <v>363.225914582146</v>
+        <v>358.796330257973</v>
       </c>
       <c r="J41" s="20" t="n">
         <f aca="false">J38*J40</f>
-        <v>376.222367410384</v>
+        <v>373.900007117728</v>
       </c>
       <c r="K41" s="20" t="n">
         <f aca="false">K38*K40</f>
@@ -2109,43 +2100,43 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B42" s="20" t="n">
         <f aca="false">B41*(1-$B$9)</f>
-        <v>164.34</v>
+        <v>159.36</v>
       </c>
       <c r="C42" s="20" t="n">
         <f aca="false">C41*(1-$B$9)</f>
-        <v>191.8545</v>
+        <v>186.1275</v>
       </c>
       <c r="D42" s="20" t="n">
         <f aca="false">D41*(1-$B$9)</f>
-        <v>217.294</v>
+        <v>210.903</v>
       </c>
       <c r="E42" s="20" t="n">
         <f aca="false">E41*(1-$B$9)</f>
-        <v>238.459</v>
+        <v>231.4455</v>
       </c>
       <c r="F42" s="20" t="n">
         <f aca="false">F41*(1-$B$9)</f>
-        <v>258.213</v>
+        <v>250.6185</v>
       </c>
       <c r="G42" s="20" t="n">
         <f aca="false">G41*(1-$B$9)</f>
-        <v>274.127620771598</v>
+        <v>267.600772657988</v>
       </c>
       <c r="H42" s="20" t="n">
         <f aca="false">H41*(1-$B$9)</f>
-        <v>288.661096361663</v>
+        <v>283.444329559946</v>
       </c>
       <c r="I42" s="20" t="n">
         <f aca="false">I41*(1-$B$9)</f>
-        <v>301.477509103181</v>
+        <v>297.800954114118</v>
       </c>
       <c r="J42" s="20" t="n">
         <f aca="false">J41*(1-$B$9)</f>
-        <v>312.264564950619</v>
+        <v>310.337005907714</v>
       </c>
       <c r="K42" s="20" t="n">
         <f aca="false">K41*(1-$B$9)</f>
@@ -2158,38 +2149,38 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B43" s="22" t="n">
-        <v>0.22</v>
+        <v>0.32</v>
       </c>
       <c r="C43" s="22" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D43" s="22" t="n">
         <v>0.17</v>
       </c>
-      <c r="D43" s="22" t="n">
-        <v>0.13</v>
-      </c>
       <c r="E43" s="22" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="F43" s="22" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="G43" s="7" t="n">
         <f aca="false">$F43+($L43-$F43)*G$17/5</f>
-        <v>0.076</v>
+        <v>0.084</v>
       </c>
       <c r="H43" s="7" t="n">
         <f aca="false">$F43+($L43-$F43)*H$17/5</f>
-        <v>0.072</v>
+        <v>0.078</v>
       </c>
       <c r="I43" s="7" t="n">
         <f aca="false">$F43+($L43-$F43)*I$17/5</f>
-        <v>0.068</v>
+        <v>0.072</v>
       </c>
       <c r="J43" s="7" t="n">
         <f aca="false">$F43+($L43-$F43)*J$17/5</f>
-        <v>0.064</v>
+        <v>0.066</v>
       </c>
       <c r="K43" s="7" t="n">
         <f aca="false">$F43+($L43-$F43)*K$17/5</f>
@@ -2201,43 +2192,43 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B44" s="20" t="n">
         <f aca="false">B38*B43</f>
-        <v>132</v>
+        <v>192</v>
       </c>
       <c r="C44" s="20" t="n">
         <f aca="false">C38*C43</f>
-        <v>117.3</v>
+        <v>165.6</v>
       </c>
       <c r="D44" s="20" t="n">
         <f aca="false">D38*D43</f>
-        <v>100.1</v>
+        <v>130.9</v>
       </c>
       <c r="E44" s="20" t="n">
         <f aca="false">E38*E43</f>
-        <v>84.5</v>
+        <v>101.4</v>
       </c>
       <c r="F44" s="20" t="n">
         <f aca="false">F38*F43</f>
-        <v>73.2</v>
+        <v>82.35</v>
       </c>
       <c r="G44" s="20" t="n">
         <f aca="false">G38*G43</f>
-        <v>74.7048880473373</v>
+        <v>82.5685604733728</v>
       </c>
       <c r="H44" s="20" t="n">
         <f aca="false">H38*H43</f>
-        <v>75.4231344826526</v>
+        <v>81.7083956895403</v>
       </c>
       <c r="I44" s="20" t="n">
         <f aca="false">I38*I43</f>
-        <v>75.3029335109327</v>
+        <v>79.7325178351052</v>
       </c>
       <c r="J44" s="20" t="n">
         <f aca="false">J38*J43</f>
-        <v>74.3155293650142</v>
+        <v>76.6378896576709</v>
       </c>
       <c r="K44" s="20" t="n">
         <f aca="false">K38*K43</f>
@@ -2250,7 +2241,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B45" s="20" t="n">
         <f aca="false">$B$11*(B38-$B$12)</f>
@@ -2299,43 +2290,43 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B46" s="20" t="n">
         <f aca="false">B42-B44-B45</f>
-        <v>32.34</v>
+        <v>-32.64</v>
       </c>
       <c r="C46" s="20" t="n">
         <f aca="false">C42-C44-C45</f>
-        <v>74.5545</v>
+        <v>20.5275</v>
       </c>
       <c r="D46" s="20" t="n">
         <f aca="false">D42-D44-D45</f>
-        <v>117.194</v>
+        <v>80.003</v>
       </c>
       <c r="E46" s="20" t="n">
         <f aca="false">E42-E44-E45</f>
-        <v>153.959</v>
+        <v>130.0455</v>
       </c>
       <c r="F46" s="20" t="n">
         <f aca="false">F42-F44-F45</f>
-        <v>185.013</v>
+        <v>168.2685</v>
       </c>
       <c r="G46" s="20" t="n">
         <f aca="false">G42-G44-G45</f>
-        <v>199.42273272426</v>
+        <v>185.032212184615</v>
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">H42-H44-H45</f>
-        <v>213.237961879011</v>
+        <v>201.735933870406</v>
       </c>
       <c r="I46" s="20" t="n">
         <f aca="false">I42-I44-I45</f>
-        <v>226.174575592248</v>
+        <v>218.068436279013</v>
       </c>
       <c r="J46" s="20" t="n">
         <f aca="false">J42-J44-J45</f>
-        <v>237.949035585605</v>
+        <v>233.699116250043</v>
       </c>
       <c r="K46" s="20" t="n">
         <f aca="false">K42-K44-K45</f>
@@ -2348,7 +2339,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B47" s="23" t="n">
         <f aca="false">1/(1+$B$10)^B$16</f>
@@ -2393,43 +2384,43 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B48" s="20" t="n">
         <f aca="false">B46*B47</f>
-        <v>30.9448890187316</v>
+        <v>-31.231947358423</v>
       </c>
       <c r="C48" s="20" t="n">
         <f aca="false">C46*C47</f>
-        <v>65.3161538989244</v>
+        <v>17.9838554233503</v>
       </c>
       <c r="D48" s="20" t="n">
         <f aca="false">D46*D47</f>
-        <v>94.0047821068751</v>
+        <v>64.1727783239443</v>
       </c>
       <c r="E48" s="20" t="n">
         <f aca="false">E46*E47</f>
-        <v>113.070022577598</v>
+        <v>95.5075547458412</v>
       </c>
       <c r="F48" s="20" t="n">
         <f aca="false">F46*F47</f>
-        <v>124.406327675249</v>
+        <v>113.147001283275</v>
       </c>
       <c r="G48" s="20" t="n">
         <f aca="false">G46*G47</f>
-        <v>122.775784006202</v>
+        <v>113.916174986827</v>
       </c>
       <c r="H48" s="20" t="n">
         <f aca="false">H46*H47</f>
-        <v>120.198875191766</v>
+        <v>113.715363452694</v>
       </c>
       <c r="I48" s="20" t="n">
         <f aca="false">I46*I47</f>
-        <v>116.72865799427</v>
+        <v>112.545080945122</v>
       </c>
       <c r="J48" s="20" t="n">
         <f aca="false">J46*J47</f>
-        <v>112.438614438807</v>
+        <v>110.430390112992</v>
       </c>
       <c r="K48" s="20" t="n">
         <f aca="false">K46*K47</f>
@@ -2439,7 +2430,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B49" s="20" t="n">
         <f aca="false">L46/($B$10-L39)</f>
@@ -2452,7 +2443,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B50" s="20" t="n">
         <f aca="false">B49/(1+$B$10)^$K$16</f>
@@ -2461,34 +2452,34 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B51" s="20" t="n">
         <f aca="false">SUM(B48:K48)+B50+$B$7+$B$8</f>
-        <v>3269.1540732165</v>
+        <v>3097.7762182237</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B52" s="24" t="n">
         <f aca="false">B51/$B$6</f>
-        <v>267.306138447792</v>
+        <v>252.467499447734</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B53" s="7" t="n">
         <f aca="false">B52/$B$4-1</f>
-        <v>-0.165893411402652</v>
+        <v>-0.215671504402951</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B55" s="19"/>
       <c r="C55" s="19"/>
@@ -2504,7 +2495,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B56" s="13" t="n">
         <v>622</v>
@@ -2548,7 +2539,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B57" s="7" t="n">
         <f aca="false">B56/$B$12-1</f>
@@ -2596,16 +2587,16 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B58" s="22" t="n">
-        <v>0.34</v>
+        <v>0.335</v>
       </c>
       <c r="C58" s="22" t="n">
-        <v>0.35</v>
+        <v>0.345</v>
       </c>
       <c r="D58" s="22" t="n">
-        <v>0.36</v>
+        <v>0.355</v>
       </c>
       <c r="E58" s="22" t="n">
         <v>0.36</v>
@@ -2639,19 +2630,19 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B59" s="20" t="n">
         <f aca="false">B56*B58</f>
-        <v>211.48</v>
+        <v>208.37</v>
       </c>
       <c r="C59" s="20" t="n">
         <f aca="false">C56*C58</f>
-        <v>255.5</v>
+        <v>251.85</v>
       </c>
       <c r="D59" s="20" t="n">
         <f aca="false">D56*D58</f>
-        <v>302.4</v>
+        <v>298.2</v>
       </c>
       <c r="E59" s="20" t="n">
         <f aca="false">E56*E58</f>
@@ -2688,19 +2679,19 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B60" s="20" t="n">
         <f aca="false">B59*(1-$B$9)</f>
-        <v>175.5284</v>
+        <v>172.9471</v>
       </c>
       <c r="C60" s="20" t="n">
         <f aca="false">C59*(1-$B$9)</f>
-        <v>212.065</v>
+        <v>209.0355</v>
       </c>
       <c r="D60" s="20" t="n">
         <f aca="false">D59*(1-$B$9)</f>
-        <v>250.992</v>
+        <v>247.506</v>
       </c>
       <c r="E60" s="20" t="n">
         <f aca="false">E59*(1-$B$9)</f>
@@ -2737,19 +2728,19 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B61" s="22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C61" s="22" t="n">
         <v>0.21</v>
       </c>
-      <c r="C61" s="22" t="n">
-        <v>0.16</v>
-      </c>
       <c r="D61" s="22" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E61" s="22" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="F61" s="22" t="n">
         <v>0.07</v>
@@ -2780,23 +2771,23 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B62" s="20" t="n">
         <f aca="false">B56*B61</f>
-        <v>130.62</v>
+        <v>186.6</v>
       </c>
       <c r="C62" s="20" t="n">
         <f aca="false">C56*C61</f>
-        <v>116.8</v>
+        <v>153.3</v>
       </c>
       <c r="D62" s="20" t="n">
         <f aca="false">D56*D61</f>
-        <v>100.8</v>
+        <v>117.6</v>
       </c>
       <c r="E62" s="20" t="n">
         <f aca="false">E56*E61</f>
-        <v>85.05</v>
+        <v>94.5</v>
       </c>
       <c r="F62" s="20" t="n">
         <f aca="false">F56*F61</f>
@@ -2829,7 +2820,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B63" s="20" t="n">
         <f aca="false">$B$11*(B56-$B$12)</f>
@@ -2878,23 +2869,23 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B64" s="20" t="n">
         <f aca="false">B60-B62-B63</f>
-        <v>44.9084</v>
+        <v>-13.6529</v>
       </c>
       <c r="C64" s="20" t="n">
         <f aca="false">C60-C62-C63</f>
-        <v>95.265</v>
+        <v>55.7355</v>
       </c>
       <c r="D64" s="20" t="n">
         <f aca="false">D60-D62-D63</f>
-        <v>150.192</v>
+        <v>129.906</v>
       </c>
       <c r="E64" s="20" t="n">
         <f aca="false">E60-E62-E63</f>
-        <v>197.316</v>
+        <v>187.866</v>
       </c>
       <c r="F64" s="20" t="n">
         <f aca="false">F60-F62-F63</f>
@@ -2927,7 +2918,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B65" s="23" t="n">
         <f aca="false">1/(1+$B$10)^B$16</f>
@@ -2972,23 +2963,23 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B66" s="20" t="n">
         <f aca="false">B64*B65</f>
-        <v>42.9711024739891</v>
+        <v>-13.0639293532418</v>
       </c>
       <c r="C66" s="20" t="n">
         <f aca="false">C64*C65</f>
-        <v>83.4603330607949</v>
+        <v>48.8290914114306</v>
       </c>
       <c r="D66" s="20" t="n">
         <f aca="false">D64*D65</f>
-        <v>120.473456270763</v>
+        <v>104.201454207346</v>
       </c>
       <c r="E66" s="20" t="n">
         <f aca="false">E64*E65</f>
-        <v>144.912116699389</v>
+        <v>137.97188122528</v>
       </c>
       <c r="F66" s="20" t="n">
         <f aca="false">F64*F65</f>
@@ -3018,7 +3009,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B67" s="20" t="n">
         <f aca="false">L64/($B$10-L57)</f>
@@ -3031,7 +3022,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B68" s="20" t="n">
         <f aca="false">B67/(1+$B$10)^$K$16</f>
@@ -3040,38 +3031,38 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B69" s="20" t="n">
         <f aca="false">SUM(B66:K66)+B68+$B$7+$B$8</f>
-        <v>4206.38322379445</v>
+        <v>4110.82471278033</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B70" s="24" t="n">
         <f aca="false">B69/$B$6</f>
-        <v>343.939756647134</v>
+        <v>335.030538938902</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B71" s="7" t="n">
         <f aca="false">B70/$B$4-1</f>
-        <v>0.0732354249918363</v>
+        <v>0.0408230729096954</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B74" s="19"/>
       <c r="C74" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D74" s="19"/>
       <c r="E74" s="19"/>
@@ -3085,68 +3076,68 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B75" s="8" t="n">
         <f aca="false">B34</f>
-        <v>149.10637041906</v>
+        <v>132.552074944012</v>
       </c>
       <c r="C75" s="7" t="n">
         <f aca="false">B75/$B$4-1</f>
-        <v>-0.534725963681281</v>
+        <v>-0.588206918686471</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B76" s="8" t="n">
         <f aca="false">B52</f>
-        <v>267.306138447792</v>
+        <v>252.467499447734</v>
       </c>
       <c r="C76" s="7" t="n">
         <f aca="false">B76/$B$4-1</f>
-        <v>-0.165893411402652</v>
+        <v>-0.215671504402951</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B77" s="8" t="n">
         <f aca="false">B70</f>
-        <v>343.939756647134</v>
+        <v>335.030538938902</v>
       </c>
       <c r="C77" s="7" t="n">
         <f aca="false">B77/$B$4-1</f>
-        <v>0.0732354249918363</v>
+        <v>0.0408230729096954</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B78" s="8" t="n">
         <f aca="false">INDEX(B34:B70,1+($B$13-1)*18)</f>
-        <v>267.306138447792</v>
+        <v>252.467499447734</v>
       </c>
       <c r="C78" s="7" t="n">
         <f aca="false">B78/$B$4-1</f>
-        <v>-0.165893411402652</v>
+        <v>-0.215671504402951</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B79" s="25" t="n">
         <f aca="false">B50/(SUM(B48:K48)+B50)</f>
-        <v>0.67996426670421</v>
+        <v>0.723573976617628</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3186,104 +3177,104 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B83" s="8" t="n">
         <f aca="false">IF(B82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+B82)^$B$16:$K$16)+$L46/(B82-$L39)/(1+B82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>1441.2536819866</v>
+        <v>1421.09956518445</v>
       </c>
       <c r="C83" s="8" t="n">
         <f aca="false">IF(C82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+C82)^$B$16:$K$16)+$L46/(C82-$L39)/(1+C82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>714.453274331295</v>
+        <v>697.04841956413</v>
       </c>
       <c r="D83" s="8" t="n">
         <f aca="false">IF(D82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+D82)^$B$16:$K$16)+$L46/(D82-$L39)/(1+D82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>472.503128387145</v>
+        <v>456.249221201014</v>
       </c>
       <c r="E83" s="8" t="n">
         <f aca="false">IF(E82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+E82)^$B$16:$K$16)+$L46/(E82-$L39)/(1+E82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>351.7520812599</v>
+        <v>336.237436641615</v>
       </c>
       <c r="F83" s="8" t="n">
         <f aca="false">IF(F82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+F82)^$B$16:$K$16)+$L46/(F82-$L39)/(1+F82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>279.470660052549</v>
+        <v>264.521734182303</v>
       </c>
       <c r="G83" s="8" t="n">
         <f aca="false">IF(G82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+G82)^$B$16:$K$16)+$L46/(G82-$L39)/(1+G82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>231.416287614912</v>
+        <v>216.939531036058</v>
       </c>
       <c r="H83" s="8" t="n">
         <f aca="false">IF(H82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+H82)^$B$16:$K$16)+$L46/(H82-$L39)/(1+H82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>197.199744767794</v>
+        <v>183.136367465769</v>
       </c>
       <c r="I83" s="8" t="n">
         <f aca="false">IF(I82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+I82)^$B$16:$K$16)+$L46/(I82-$L39)/(1+I82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>171.626789194869</v>
+        <v>157.935758287194</v>
       </c>
       <c r="J83" s="8" t="n">
         <f aca="false">IF(J82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+J82)^$B$16:$K$16)+$L46/(J82-$L39)/(1+J82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>151.812031063774</v>
+        <v>138.462483005197</v>
       </c>
       <c r="K83" s="8" t="n">
         <f aca="false">IF(K82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+K82)^$B$16:$K$16)+$L46/(K82-$L39)/(1+K82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>136.024485420205</v>
+        <v>122.991906920388</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B84" s="7" t="n">
         <f aca="false">IFERROR(B83/$B$4-1,"n/a")</f>
-        <v>3.4973123287253</v>
+        <v>3.41486086919274</v>
       </c>
       <c r="C84" s="7" t="n">
         <f aca="false">IFERROR(C83/$B$4-1,"n/a")</f>
-        <v>1.22939206269322</v>
+        <v>1.16548640704629</v>
       </c>
       <c r="D84" s="7" t="n">
         <f aca="false">IFERROR(D83/$B$4-1,"n/a")</f>
-        <v>0.47440674130853</v>
+        <v>0.417407254655362</v>
       </c>
       <c r="E84" s="7" t="n">
         <f aca="false">IFERROR(E83/$B$4-1,"n/a")</f>
-        <v>0.0976131346456775</v>
+        <v>0.0445724832756991</v>
       </c>
       <c r="F84" s="7" t="n">
         <f aca="false">IFERROR(F83/$B$4-1,"n/a")</f>
-        <v>-0.127935032756425</v>
+        <v>-0.178223199905859</v>
       </c>
       <c r="G84" s="7" t="n">
         <f aca="false">IFERROR(G83/$B$4-1,"n/a")</f>
-        <v>-0.277884708038467</v>
+        <v>-0.32604451509504</v>
       </c>
       <c r="H84" s="7" t="n">
         <f aca="false">IFERROR(H83/$B$4-1,"n/a")</f>
-        <v>-0.384654586177195</v>
+        <v>-0.431059158514494</v>
       </c>
       <c r="I84" s="7" t="n">
         <f aca="false">IFERROR(I83/$B$4-1,"n/a")</f>
-        <v>-0.464452868615256</v>
+        <v>-0.509348664801038</v>
       </c>
       <c r="J84" s="7" t="n">
         <f aca="false">IFERROR(J83/$B$4-1,"n/a")</f>
-        <v>-0.526283174513139</v>
+        <v>-0.56984534156017</v>
       </c>
       <c r="K84" s="7" t="n">
         <f aca="false">IFERROR(K83/$B$4-1,"n/a")</f>
-        <v>-0.575546898554608</v>
+        <v>-0.617907027492658</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B86" s="26" t="n">
         <f aca="false">IFERROR(IF(MATCH($B$4,$B$83:$K$83,-1)=10,"above 14%",INDEX($B$82:$K$82,MATCH($B$4,$B$83:$K$83,-1))+(INDEX($B$83:$K$83,MATCH($B$4,$B$83:$K$83,-1))-$B$4)/(INDEX($B$83:$K$83,MATCH($B$4,$B$83:$K$83,-1))-INDEX($B$83:$K$83,MATCH($B$4,$B$83:$K$83,-1)+1))*(INDEX($B$82:$K$82,MATCH($B$4,$B$83:$K$83,-1)+1)-INDEX($B$82:$K$82,MATCH($B$4,$B$83:$K$83,-1)))),"below 5%")</f>
-        <v>0.0843278176794784</v>
+        <v>0.082000599052872</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -3312,163 +3303,163 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B6" s="16" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>0.0503</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>0.05</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>0.012</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
         <v>98</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B13" s="27" t="n">
         <v>1.21</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B15" s="28" t="n">
         <f aca="false">0.67*IF(ISNUMBER(B14),B14,B13)+0.33</f>
         <v>1.1407</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B16" s="28" t="n">
         <f aca="false">IF($B$6=1,IF(ISNUMBER(B14),B14,B13),B15)</f>
         <v>1.1407</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B17" s="25" t="n">
         <f aca="false">$B$7+B16*$B$8</f>
         <v>0.107335</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B18" s="25" t="n">
         <f aca="false">$B$7+$B$9</f>
         <v>0.0623</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">GOOG!B9</f>
         <v>0.17</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B20" s="25" t="n">
         <f aca="false">B18*(1-B19)</f>
@@ -3478,85 +3469,85 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B21" s="29" t="n">
         <f aca="false">GOOG!B4*GOOG!B6</f>
-        <v>3919.3481</v>
+        <v>3949.5903</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" s="30" t="n">
+        <v>125.1</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="B22" s="30" t="n">
-        <v>120.79</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B23" s="25" t="n">
         <f aca="false">B21/(B21+B22)</f>
-        <v>0.970102507139546</v>
+        <v>0.969298280166225</v>
       </c>
       <c r="C23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B24" s="25" t="n">
         <f aca="false">B22/(B21+B22)</f>
-        <v>0.0298974928604544</v>
+        <v>0.0307017198337749</v>
       </c>
       <c r="C24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B25" s="25" t="n">
         <f aca="false">B23*B17+B24*B20</f>
-        <v>0.105671922062144</v>
+        <v>0.105627186132526</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B26" s="31" t="n">
         <v>0.0922</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B27" s="26" t="n">
         <f aca="false">IF($B$5=1,B25,B26)</f>
         <v>0.0922</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B28" s="1" t="str">
         <f aca="false">IF(B27&gt;MAX(GOOG!L21,GOOG!L39,GOOG!L57),"OK","WACC must exceed growth")</f>
@@ -3566,14 +3557,14 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B29" s="25" t="n">
         <f aca="false">B27</f>
         <v>0.0922</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>